<commit_message>
feat: staff identity, page access control, farm operations analytics, and daily activity log edit action
</commit_message>
<xml_diff>
--- a/Farm Management  Data Records.xlsx
+++ b/Farm Management  Data Records.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benedictasante/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Farm Actual Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8344311-5454-BD42-B555-E0C112D5E73C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA05E7B4-255B-4492-B264-666292768127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{7B054ADF-9E21-634C-B6C3-26E0C5B37783}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7B054ADF-9E21-634C-B6C3-26E0C5B37783}"/>
   </bookViews>
   <sheets>
     <sheet name="FARMS  (2)" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="210">
   <si>
     <t xml:space="preserve">GRAND TOTAL </t>
   </si>
@@ -657,6 +657,18 @@
   </si>
   <si>
     <t>Price 2026</t>
+  </si>
+  <si>
+    <t>Tracking this section</t>
+  </si>
+  <si>
+    <t>Knowlede base(chemicals needed for the activites)</t>
+  </si>
+  <si>
+    <t>Activites</t>
+  </si>
+  <si>
+    <t>Things needed</t>
   </si>
 </sst>
 </file>
@@ -664,15 +676,15 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="9">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="167" formatCode="_([$GHS]\ * #,##0_);_([$GHS]\ * \(#,##0\);_([$GHS]\ * &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_([$$-409]* #,##0_);_([$$-409]* \(#,##0\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="170" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="169" formatCode="_([$GHS]\ * #,##0_);_([$GHS]\ * \(#,##0\);_([$GHS]\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="170" formatCode="_([$$-409]* #,##0_);_([$$-409]* \(#,##0\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="171" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="172" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -828,7 +840,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -1150,24 +1162,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1178,20 +1199,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1203,7 +1224,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1221,14 +1242,14 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="8" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1237,26 +1258,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1264,43 +1273,28 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1308,19 +1302,19 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="44" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1329,18 +1323,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1387,25 +1381,61 @@
     <xf numFmtId="0" fontId="2" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1413,7 +1443,7 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1725,37 +1755,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B795C603-F572-E747-AF13-070966F62982}">
-  <dimension ref="B3:CJ48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="B1:CJ48"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.1640625" customWidth="1"/>
-    <col min="2" max="2" width="21.5" customWidth="1"/>
-    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.109375" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" customWidth="1"/>
+    <col min="3" max="3" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.5" customWidth="1"/>
-    <col min="7" max="7" width="3.5" customWidth="1"/>
+    <col min="6" max="6" width="5.44140625" customWidth="1"/>
+    <col min="7" max="7" width="3.44140625" customWidth="1"/>
     <col min="8" max="8" width="3.33203125" customWidth="1"/>
     <col min="9" max="9" width="17.33203125" customWidth="1"/>
     <col min="10" max="10" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="5.6640625" customWidth="1"/>
-    <col min="12" max="12" width="4.5" customWidth="1"/>
-    <col min="13" max="13" width="8.5" customWidth="1"/>
-    <col min="14" max="14" width="14.1640625" customWidth="1"/>
-    <col min="15" max="15" width="18.1640625" customWidth="1"/>
-    <col min="16" max="16" width="11.83203125" customWidth="1"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1"/>
-    <col min="18" max="18" width="8.5" customWidth="1"/>
+    <col min="12" max="12" width="4.44140625" customWidth="1"/>
+    <col min="13" max="13" width="8.44140625" customWidth="1"/>
+    <col min="14" max="14" width="14.109375" customWidth="1"/>
+    <col min="15" max="15" width="18.109375" customWidth="1"/>
+    <col min="16" max="16" width="11.77734375" customWidth="1"/>
+    <col min="17" max="17" width="7.77734375" customWidth="1"/>
+    <col min="18" max="18" width="8.44140625" customWidth="1"/>
     <col min="19" max="19" width="13.6640625" customWidth="1"/>
-    <col min="20" max="20" width="13.83203125" customWidth="1"/>
+    <col min="20" max="20" width="13.77734375" customWidth="1"/>
     <col min="21" max="21" width="15.6640625" customWidth="1"/>
-    <col min="22" max="22" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.109375" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="14.33203125" customWidth="1"/>
     <col min="24" max="24" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="8.33203125" customWidth="1"/>
-    <col min="28" max="30" width="5.1640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="30" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="23" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="20" customWidth="1"/>
     <col min="37" max="37" width="22" customWidth="1"/>
@@ -1763,242 +1793,268 @@
     <col min="40" max="40" width="41" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="5.44140625" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="11.33203125" customWidth="1"/>
-    <col min="45" max="45" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="9" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="5.83203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="5.77734375" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="57" max="57" width="11" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="11.1640625" customWidth="1"/>
+    <col min="58" max="58" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="11.109375" customWidth="1"/>
     <col min="60" max="60" width="13" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="62" max="62" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="6.83203125" customWidth="1"/>
-    <col min="70" max="70" width="14.83203125" customWidth="1"/>
+    <col min="63" max="63" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="6.77734375" customWidth="1"/>
+    <col min="70" max="70" width="14.77734375" customWidth="1"/>
     <col min="74" max="74" width="9.6640625" customWidth="1"/>
+    <col min="78" max="78" width="34.88671875" customWidth="1"/>
+    <col min="79" max="79" width="34.5546875" customWidth="1"/>
+    <col min="80" max="80" width="19.109375" customWidth="1"/>
+    <col min="82" max="82" width="19.33203125" customWidth="1"/>
+    <col min="83" max="83" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:88" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:88" x14ac:dyDescent="0.3">
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
+    </row>
+    <row r="2" spans="2:88" x14ac:dyDescent="0.3">
+      <c r="N2" s="116"/>
+      <c r="O2" s="116"/>
+    </row>
+    <row r="3" spans="2:88" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="N3" s="116"/>
+      <c r="O3" s="116"/>
       <c r="S3" s="12"/>
       <c r="X3" t="s">
         <v>205</v>
       </c>
+      <c r="AN3" s="117" t="s">
+        <v>206</v>
+      </c>
+      <c r="AO3" s="117"/>
+      <c r="AP3" s="117"/>
+      <c r="AQ3" s="117"/>
+      <c r="AR3" s="117"/>
+      <c r="AS3" s="117"/>
+      <c r="AT3" s="117"/>
+      <c r="AU3" s="117"/>
+      <c r="AV3" s="117"/>
       <c r="BO3" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="4" spans="2:88" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="111" t="s">
+    <row r="4" spans="2:88" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="103" t="s">
         <v>203</v>
       </c>
-      <c r="C4" s="110"/>
-      <c r="D4" s="110"/>
-      <c r="E4" s="110"/>
-      <c r="F4" s="109"/>
-      <c r="I4" s="115" t="s">
+      <c r="C4" s="104"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="105"/>
+      <c r="I4" s="106" t="s">
         <v>202</v>
       </c>
-      <c r="J4" s="114"/>
-      <c r="K4" s="113"/>
-      <c r="L4" s="113"/>
-      <c r="M4" s="112"/>
+      <c r="J4" s="107"/>
+      <c r="K4" s="108"/>
+      <c r="L4" s="108"/>
+      <c r="M4" s="109"/>
       <c r="N4" s="12"/>
-      <c r="O4" s="111" t="s">
+      <c r="O4" s="103" t="s">
         <v>201</v>
       </c>
-      <c r="P4" s="110"/>
-      <c r="Q4" s="110"/>
-      <c r="R4" s="109"/>
+      <c r="P4" s="104"/>
+      <c r="Q4" s="104"/>
+      <c r="R4" s="105"/>
       <c r="S4" s="12"/>
-      <c r="T4" s="108" t="s">
+      <c r="T4" s="99" t="s">
         <v>193</v>
       </c>
-      <c r="U4" s="108" t="s">
+      <c r="U4" s="99" t="s">
         <v>168</v>
       </c>
-      <c r="V4" s="108" t="s">
+      <c r="V4" s="99" t="s">
         <v>200</v>
       </c>
-      <c r="W4" s="108" t="s">
+      <c r="W4" s="99" t="s">
         <v>199</v>
       </c>
-      <c r="X4" s="108">
+      <c r="X4" s="99">
         <v>5.22</v>
       </c>
-      <c r="Z4" s="107" t="s">
+      <c r="Z4" s="98" t="s">
         <v>198</v>
       </c>
-      <c r="AA4" s="106">
+      <c r="AA4" s="97">
         <v>2026</v>
       </c>
-      <c r="AB4" s="105">
+      <c r="AB4" s="96">
         <v>2027</v>
       </c>
-      <c r="AC4" s="105">
+      <c r="AC4" s="96">
         <v>2028</v>
       </c>
-      <c r="AD4" s="105">
+      <c r="AD4" s="96">
         <v>2029</v>
       </c>
-      <c r="AE4" s="104">
+      <c r="AE4" s="95">
         <v>2030</v>
       </c>
-      <c r="AG4" s="103"/>
-      <c r="AH4" s="103" t="s">
+      <c r="AG4" s="94"/>
+      <c r="AH4" s="94" t="s">
         <v>197</v>
       </c>
-      <c r="AI4" s="103" t="s">
+      <c r="AI4" s="94" t="s">
         <v>196</v>
       </c>
-      <c r="AJ4" s="103" t="s">
+      <c r="AJ4" s="94" t="s">
         <v>138</v>
       </c>
-      <c r="AK4" s="102" t="s">
+      <c r="AK4" s="93" t="s">
         <v>195</v>
       </c>
-      <c r="AM4" s="101" t="s">
+      <c r="AM4" s="92" t="s">
         <v>194</v>
       </c>
-      <c r="AN4" s="100" t="s">
+      <c r="AN4" s="91" t="s">
         <v>193</v>
       </c>
-      <c r="AO4" s="100" t="s">
+      <c r="AO4" s="91" t="s">
         <v>192</v>
       </c>
-      <c r="AP4" s="100" t="s">
+      <c r="AP4" s="91" t="s">
         <v>191</v>
       </c>
-      <c r="AQ4" s="100" t="s">
+      <c r="AQ4" s="91" t="s">
         <v>190</v>
       </c>
-      <c r="AR4" s="100" t="s">
+      <c r="AR4" s="91" t="s">
         <v>189</v>
       </c>
-      <c r="AS4" s="100" t="s">
+      <c r="AS4" s="91" t="s">
         <v>188</v>
       </c>
-      <c r="AT4" s="100" t="s">
+      <c r="AT4" s="91" t="s">
         <v>187</v>
       </c>
-      <c r="AU4" s="100" t="s">
+      <c r="AU4" s="91" t="s">
         <v>186</v>
       </c>
-      <c r="AV4" s="100" t="s">
+      <c r="AV4" s="91" t="s">
         <v>185</v>
       </c>
-      <c r="AW4" s="99" t="s">
+      <c r="AW4" s="90" t="s">
         <v>184</v>
       </c>
-      <c r="AZ4" s="96" t="s">
+      <c r="AZ4" s="87" t="s">
         <v>156</v>
       </c>
-      <c r="BA4" s="96" t="s">
+      <c r="BA4" s="87" t="s">
         <v>183</v>
       </c>
-      <c r="BB4" s="96" t="s">
+      <c r="BB4" s="87" t="s">
         <v>182</v>
       </c>
-      <c r="BC4" s="98" t="s">
+      <c r="BC4" s="89" t="s">
         <v>181</v>
       </c>
-      <c r="BD4" s="96" t="s">
+      <c r="BD4" s="87" t="s">
         <v>180</v>
       </c>
-      <c r="BE4" s="96" t="s">
+      <c r="BE4" s="87" t="s">
         <v>179</v>
       </c>
-      <c r="BF4" s="96" t="s">
+      <c r="BF4" s="87" t="s">
         <v>178</v>
       </c>
-      <c r="BG4" s="96" t="s">
+      <c r="BG4" s="87" t="s">
         <v>177</v>
       </c>
-      <c r="BH4" s="98" t="s">
+      <c r="BH4" s="89" t="s">
         <v>176</v>
       </c>
-      <c r="BI4" s="97" t="s">
+      <c r="BI4" s="88" t="s">
         <v>175</v>
       </c>
-      <c r="BJ4" s="96" t="s">
+      <c r="BJ4" s="87" t="s">
         <v>168</v>
       </c>
-      <c r="BL4" s="95">
+      <c r="BL4" s="86">
         <v>0.05</v>
       </c>
-      <c r="BM4" s="94" t="s">
+      <c r="BM4" s="85" t="s">
         <v>174</v>
       </c>
-      <c r="BN4" s="94" t="s">
+      <c r="BN4" s="85" t="s">
         <v>173</v>
       </c>
-      <c r="BO4" s="94" t="s">
+      <c r="BO4" s="85" t="s">
         <v>172</v>
       </c>
-      <c r="BP4" s="94" t="s">
+      <c r="BP4" s="85" t="s">
         <v>171</v>
       </c>
       <c r="BQ4" s="5"/>
-      <c r="BR4" s="93" t="s">
+      <c r="BR4" s="84" t="s">
         <v>170</v>
       </c>
-      <c r="BT4" s="92" t="s">
+      <c r="BT4" s="83" t="s">
         <v>169</v>
       </c>
-      <c r="BU4" s="92" t="s">
+      <c r="BU4" s="83" t="s">
         <v>168</v>
       </c>
-      <c r="BV4" s="91" t="s">
+      <c r="BV4" s="82" t="s">
         <v>167</v>
       </c>
-      <c r="BY4" s="90" t="s">
+      <c r="BY4" s="81" t="s">
         <v>156</v>
       </c>
-      <c r="BZ4" s="90" t="s">
+      <c r="BZ4" s="81" t="s">
         <v>166</v>
       </c>
-      <c r="CA4" s="90" t="s">
+      <c r="CA4" s="81" t="s">
         <v>165</v>
       </c>
-      <c r="CB4" s="90" t="s">
+      <c r="CB4" s="81" t="s">
         <v>164</v>
       </c>
-      <c r="CC4" s="90" t="s">
+      <c r="CC4" s="81" t="s">
         <v>163</v>
       </c>
-      <c r="CD4" s="90" t="s">
+      <c r="CD4" s="81" t="s">
         <v>162</v>
       </c>
-      <c r="CE4" s="90" t="s">
+      <c r="CE4" s="81" t="s">
         <v>161</v>
       </c>
-      <c r="CF4" s="90" t="s">
+      <c r="CF4" s="81" t="s">
         <v>160</v>
       </c>
-      <c r="CG4" s="90" t="s">
+      <c r="CG4" s="81" t="s">
         <v>159</v>
       </c>
-      <c r="CH4" s="90" t="s">
+      <c r="CH4" s="81" t="s">
         <v>158</v>
       </c>
-      <c r="CI4" s="89" t="s">
+      <c r="CI4" s="80" t="s">
         <v>157</v>
       </c>
-      <c r="CJ4" s="88">
+      <c r="CJ4" s="79">
         <f>SUM(CF5:CF153)</f>
         <v>3630</v>
       </c>
     </row>
-    <row r="5" spans="2:88" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
       <c r="D5" s="22" t="s">
@@ -2007,23 +2063,27 @@
       <c r="E5" s="22"/>
       <c r="F5" s="22"/>
       <c r="I5" s="22"/>
-      <c r="J5" s="81"/>
+      <c r="J5" s="72"/>
       <c r="K5" s="22"/>
       <c r="L5" s="22"/>
       <c r="M5" s="22"/>
       <c r="N5" s="12"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
+      <c r="O5" s="22" t="s">
+        <v>208</v>
+      </c>
+      <c r="P5" s="22" t="s">
+        <v>209</v>
+      </c>
       <c r="Q5" s="22"/>
       <c r="R5" s="22"/>
       <c r="S5" s="12"/>
-      <c r="T5" s="87" t="s">
+      <c r="T5" s="78" t="s">
         <v>155</v>
       </c>
-      <c r="U5" s="52">
+      <c r="U5" s="47">
         <v>38</v>
       </c>
-      <c r="V5" s="52" t="s">
+      <c r="V5" s="47" t="s">
         <v>122</v>
       </c>
       <c r="W5" s="1"/>
@@ -2031,10 +2091,10 @@
         <f>U5*X4</f>
         <v>198.35999999999999</v>
       </c>
-      <c r="Z5" s="71" t="s">
+      <c r="Z5" s="62" t="s">
         <v>154</v>
       </c>
-      <c r="AA5" s="70">
+      <c r="AA5" s="61">
         <v>3000</v>
       </c>
       <c r="AB5">
@@ -2046,25 +2106,25 @@
       <c r="AD5">
         <v>8000</v>
       </c>
-      <c r="AE5" s="68">
+      <c r="AE5" s="59">
         <v>100000</v>
       </c>
-      <c r="AG5" s="51" t="s">
+      <c r="AG5" s="110" t="s">
         <v>153</v>
       </c>
-      <c r="AH5" s="80" t="s">
+      <c r="AH5" s="71" t="s">
         <v>152</v>
       </c>
-      <c r="AI5" s="50" t="s">
+      <c r="AI5" s="46" t="s">
         <v>151</v>
       </c>
-      <c r="AJ5" s="50" t="s">
+      <c r="AJ5" s="46" t="s">
         <v>150</v>
       </c>
-      <c r="AK5" s="49" t="s">
+      <c r="AK5" s="45" t="s">
         <v>149</v>
       </c>
-      <c r="AM5" s="86" t="s">
+      <c r="AM5" s="77" t="s">
         <v>148</v>
       </c>
       <c r="AN5" s="32" t="s">
@@ -2097,48 +2157,48 @@
         <v>527</v>
       </c>
       <c r="BC5" s="31"/>
-      <c r="BD5" s="76">
+      <c r="BD5" s="67">
         <v>9845</v>
       </c>
       <c r="BE5" s="13"/>
-      <c r="BF5" s="76">
+      <c r="BF5" s="67">
         <v>956</v>
       </c>
-      <c r="BG5" s="75">
+      <c r="BG5" s="66">
         <f>BF5/BD5</f>
         <v>9.7105129507364149E-2</v>
       </c>
-      <c r="BH5" s="64">
+      <c r="BH5" s="58">
         <f>BD5-BF5</f>
         <v>8889</v>
       </c>
-      <c r="BI5" s="63">
+      <c r="BI5" s="57">
         <v>5.25</v>
       </c>
-      <c r="BJ5" s="43">
+      <c r="BJ5" s="42">
         <f>BH5*BI5</f>
         <v>46667.25</v>
       </c>
-      <c r="BK5" s="72"/>
-      <c r="BL5" s="74">
+      <c r="BK5" s="63"/>
+      <c r="BL5" s="65">
         <f>BJ5*0.05</f>
         <v>2333.3625000000002</v>
       </c>
-      <c r="BM5" s="74">
+      <c r="BM5" s="65">
         <v>120</v>
       </c>
-      <c r="BN5" s="85">
+      <c r="BN5" s="76">
         <v>240</v>
       </c>
-      <c r="BO5" s="85">
+      <c r="BO5" s="76">
         <v>900</v>
       </c>
-      <c r="BP5" s="73">
+      <c r="BP5" s="64">
         <f>SUM(BL5:BO5)</f>
         <v>3593.3625000000002</v>
       </c>
-      <c r="BQ5" s="61"/>
-      <c r="BR5" s="84">
+      <c r="BQ5" s="55"/>
+      <c r="BR5" s="75">
         <f>BJ5-BP5</f>
         <v>43073.887499999997</v>
       </c>
@@ -2152,27 +2212,27 @@
       <c r="BY5" s="34">
         <v>45874</v>
       </c>
-      <c r="BZ5" s="82" t="s">
+      <c r="BZ5" s="73" t="s">
         <v>144</v>
       </c>
-      <c r="CA5" s="82" t="s">
+      <c r="CA5" s="73" t="s">
         <v>143</v>
       </c>
-      <c r="CB5" s="82" t="s">
+      <c r="CB5" s="73" t="s">
         <v>142</v>
       </c>
-      <c r="CC5" s="82"/>
-      <c r="CD5" s="82"/>
-      <c r="CE5" s="82"/>
-      <c r="CF5" s="83">
+      <c r="CC5" s="73"/>
+      <c r="CD5" s="73"/>
+      <c r="CE5" s="73"/>
+      <c r="CF5" s="74">
         <v>800</v>
       </c>
-      <c r="CG5" s="82"/>
-      <c r="CH5" s="82"/>
-      <c r="CI5" s="82"/>
-      <c r="CJ5" s="82"/>
-    </row>
-    <row r="6" spans="2:88" x14ac:dyDescent="0.2">
+      <c r="CG5" s="73"/>
+      <c r="CH5" s="73"/>
+      <c r="CI5" s="73"/>
+      <c r="CJ5" s="73"/>
+    </row>
+    <row r="6" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>141</v>
       </c>
@@ -2187,7 +2247,7 @@
       <c r="I6" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="J6" s="81">
+      <c r="J6" s="72">
         <v>46113</v>
       </c>
       <c r="K6" s="22">
@@ -2217,7 +2277,7 @@
         <f>10*U5</f>
         <v>380</v>
       </c>
-      <c r="V6" s="52" t="s">
+      <c r="V6" s="47" t="s">
         <v>122</v>
       </c>
       <c r="W6" s="1"/>
@@ -2225,10 +2285,10 @@
         <f>U6*X4</f>
         <v>1983.6</v>
       </c>
-      <c r="Z6" s="71" t="s">
+      <c r="Z6" s="62" t="s">
         <v>135</v>
       </c>
-      <c r="AA6" s="70">
+      <c r="AA6" s="61">
         <v>5</v>
       </c>
       <c r="AB6">
@@ -2240,20 +2300,20 @@
       <c r="AD6">
         <v>20</v>
       </c>
-      <c r="AE6" s="68">
+      <c r="AE6" s="59">
         <v>30</v>
       </c>
-      <c r="AG6" s="51"/>
-      <c r="AH6" s="80" t="s">
+      <c r="AG6" s="110"/>
+      <c r="AH6" s="71" t="s">
         <v>134</v>
       </c>
-      <c r="AI6" s="50" t="s">
+      <c r="AI6" s="46" t="s">
         <v>133</v>
       </c>
-      <c r="AJ6" s="50" t="s">
+      <c r="AJ6" s="46" t="s">
         <v>132</v>
       </c>
-      <c r="AK6" s="49" t="s">
+      <c r="AK6" s="45" t="s">
         <v>131</v>
       </c>
       <c r="AM6" s="28" t="s">
@@ -2291,43 +2351,43 @@
       <c r="BC6" s="31">
         <v>0</v>
       </c>
-      <c r="BD6" s="76">
+      <c r="BD6" s="67">
         <v>9893</v>
       </c>
       <c r="BE6" s="13">
         <v>0</v>
       </c>
-      <c r="BF6" s="76">
+      <c r="BF6" s="67">
         <v>769</v>
       </c>
-      <c r="BG6" s="75">
+      <c r="BG6" s="66">
         <f>BF6/BD6</f>
         <v>7.7731729505711111E-2</v>
       </c>
-      <c r="BH6" s="64">
+      <c r="BH6" s="58">
         <f>BD6-BF6</f>
         <v>9124</v>
       </c>
-      <c r="BI6" s="63">
+      <c r="BI6" s="57">
         <v>5.25</v>
       </c>
-      <c r="BJ6" s="43">
+      <c r="BJ6" s="42">
         <f>BH6*BI6</f>
         <v>47901</v>
       </c>
-      <c r="BK6" s="72"/>
-      <c r="BL6" s="74">
+      <c r="BK6" s="63"/>
+      <c r="BL6" s="65">
         <f>BJ6*0.05</f>
         <v>2395.0500000000002</v>
       </c>
-      <c r="BM6" s="79"/>
-      <c r="BN6" s="79"/>
-      <c r="BO6" s="79"/>
-      <c r="BP6" s="73">
+      <c r="BM6" s="70"/>
+      <c r="BN6" s="70"/>
+      <c r="BO6" s="70"/>
+      <c r="BP6" s="64">
         <f>SUM(BL6:BO6)</f>
         <v>2395.0500000000002</v>
       </c>
-      <c r="BR6" s="78"/>
+      <c r="BR6" s="69"/>
       <c r="BT6" s="1" t="s">
         <v>128</v>
       </c>
@@ -2351,7 +2411,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="7" spans="2:88" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:88" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>112</v>
       </c>
@@ -2366,7 +2426,7 @@
       <c r="I7" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="J7" s="42">
+      <c r="J7" s="41">
         <v>46113</v>
       </c>
       <c r="K7" s="1">
@@ -2394,7 +2454,7 @@
         <f>U6*24</f>
         <v>9120</v>
       </c>
-      <c r="V7" s="52" t="s">
+      <c r="V7" s="47" t="s">
         <v>122</v>
       </c>
       <c r="W7" s="1"/>
@@ -2402,10 +2462,10 @@
         <f>U7*X4</f>
         <v>47606.399999999994</v>
       </c>
-      <c r="Z7" s="71" t="s">
+      <c r="Z7" s="62" t="s">
         <v>121</v>
       </c>
-      <c r="AA7" s="70">
+      <c r="AA7" s="61">
         <v>3</v>
       </c>
       <c r="AB7">
@@ -2417,11 +2477,11 @@
       <c r="AD7">
         <v>24</v>
       </c>
-      <c r="AE7" s="68">
+      <c r="AE7" s="59">
         <v>50</v>
       </c>
-      <c r="AG7" s="41"/>
-      <c r="AH7" s="77" t="s">
+      <c r="AG7" s="111"/>
+      <c r="AH7" s="68" t="s">
         <v>120</v>
       </c>
       <c r="AI7" s="40" t="s">
@@ -2465,37 +2525,37 @@
         <v>682</v>
       </c>
       <c r="BC7" s="31"/>
-      <c r="BD7" s="76">
+      <c r="BD7" s="67">
         <v>9585</v>
       </c>
       <c r="BE7" s="13"/>
-      <c r="BF7" s="76">
+      <c r="BF7" s="67">
         <v>880</v>
       </c>
-      <c r="BG7" s="75">
+      <c r="BG7" s="66">
         <f>BF7/BD7</f>
         <v>9.1810119979134061E-2</v>
       </c>
-      <c r="BH7" s="64">
+      <c r="BH7" s="58">
         <f>BD7-BF7</f>
         <v>8705</v>
       </c>
-      <c r="BI7" s="63">
+      <c r="BI7" s="57">
         <v>5.25</v>
       </c>
-      <c r="BJ7" s="43">
+      <c r="BJ7" s="42">
         <f>BH7*BI7</f>
         <v>45701.25</v>
       </c>
-      <c r="BL7" s="74">
+      <c r="BL7" s="65">
         <f>BJ7*0.05</f>
         <v>2285.0625</v>
       </c>
-      <c r="BP7" s="73">
+      <c r="BP7" s="64">
         <f>SUM(BL7:BO7)</f>
         <v>2285.0625</v>
       </c>
-      <c r="BR7" s="72">
+      <c r="BR7" s="63">
         <f>SUM(BR5:BR6)</f>
         <v>43073.887499999997</v>
       </c>
@@ -2522,7 +2582,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="2:88" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:88" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>112</v>
       </c>
@@ -2551,32 +2611,32 @@
       <c r="S8" s="12"/>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
-      <c r="V8" s="52"/>
+      <c r="V8" s="47"/>
       <c r="W8" s="1"/>
       <c r="X8" s="21"/>
-      <c r="Z8" s="71" t="s">
+      <c r="Z8" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="AA8" s="70">
+      <c r="AA8" s="61">
         <v>5</v>
       </c>
       <c r="AB8">
         <v>10</v>
       </c>
-      <c r="AC8" s="69">
+      <c r="AC8" s="60">
         <v>15</v>
       </c>
       <c r="AD8">
         <v>20</v>
       </c>
-      <c r="AE8" s="68">
+      <c r="AE8" s="59">
         <v>25</v>
       </c>
-      <c r="AG8" s="67"/>
-      <c r="AH8" s="66"/>
-      <c r="AI8" s="66"/>
-      <c r="AJ8" s="66"/>
-      <c r="AK8" s="65"/>
+      <c r="AG8" s="112"/>
+      <c r="AH8" s="113"/>
+      <c r="AI8" s="113"/>
+      <c r="AJ8" s="113"/>
+      <c r="AK8" s="114"/>
       <c r="AM8" s="28" t="s">
         <v>108</v>
       </c>
@@ -2608,16 +2668,16 @@
       <c r="BE8" s="13"/>
       <c r="BF8" s="13"/>
       <c r="BG8" s="13"/>
-      <c r="BH8" s="64">
+      <c r="BH8" s="58">
         <f>BJ8/BI8</f>
         <v>0</v>
       </c>
-      <c r="BI8" s="63">
+      <c r="BI8" s="57">
         <v>5.25</v>
       </c>
-      <c r="BJ8" s="43"/>
-      <c r="BL8" s="62"/>
-      <c r="BP8" s="61"/>
+      <c r="BJ8" s="42"/>
+      <c r="BL8" s="56"/>
+      <c r="BP8" s="55"/>
       <c r="BT8" s="1" t="s">
         <v>106</v>
       </c>
@@ -2641,7 +2701,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="9" spans="2:88" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:88" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>103</v>
       </c>
@@ -2669,40 +2729,40 @@
       <c r="T9" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="U9" s="52">
+      <c r="U9" s="47">
         <v>4</v>
       </c>
-      <c r="V9" s="52"/>
+      <c r="V9" s="47"/>
       <c r="W9" s="1"/>
       <c r="X9" s="21">
         <f>X7*U9</f>
         <v>190425.59999999998</v>
       </c>
-      <c r="Z9" s="60" t="s">
+      <c r="Z9" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="AA9" s="59">
+      <c r="AA9" s="53">
         <v>5</v>
       </c>
-      <c r="AB9" s="58">
+      <c r="AB9" s="52">
         <v>10</v>
       </c>
-      <c r="AC9" s="58">
+      <c r="AC9" s="52">
         <v>12</v>
       </c>
-      <c r="AD9" s="58">
+      <c r="AD9" s="52">
         <v>24</v>
       </c>
-      <c r="AE9" s="57">
+      <c r="AE9" s="51">
         <v>60</v>
       </c>
-      <c r="AG9" s="56" t="s">
+      <c r="AG9" s="115" t="s">
         <v>99</v>
       </c>
-      <c r="AH9" s="55"/>
-      <c r="AI9" s="55"/>
-      <c r="AJ9" s="55"/>
-      <c r="AK9" s="54"/>
+      <c r="AH9" s="50"/>
+      <c r="AI9" s="50"/>
+      <c r="AJ9" s="50"/>
+      <c r="AK9" s="49"/>
       <c r="AM9" s="25" t="s">
         <v>98</v>
       </c>
@@ -2737,7 +2797,7 @@
       <c r="BH9" s="13"/>
       <c r="BI9" s="13"/>
       <c r="BJ9" s="13"/>
-      <c r="BP9" s="53">
+      <c r="BP9" s="48">
         <f>SUM(BP5:BP8)</f>
         <v>8273.4750000000004</v>
       </c>
@@ -2763,7 +2823,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="2:88" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>4</v>
       </c>
@@ -2776,7 +2836,7 @@
       <c r="I10" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="42">
+      <c r="J10" s="41">
         <v>46113</v>
       </c>
       <c r="K10" s="1">
@@ -2797,49 +2857,49 @@
       <c r="S10" s="12"/>
       <c r="T10" s="1"/>
       <c r="U10" s="21"/>
-      <c r="V10" s="52"/>
+      <c r="V10" s="47"/>
       <c r="W10" s="14"/>
       <c r="X10" s="1"/>
-      <c r="AG10" s="51"/>
-      <c r="AH10" s="50" t="s">
+      <c r="AG10" s="110"/>
+      <c r="AH10" s="46" t="s">
         <v>93</v>
       </c>
-      <c r="AI10" s="50" t="s">
+      <c r="AI10" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="AJ10" s="50" t="s">
+      <c r="AJ10" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="AK10" s="49" t="s">
+      <c r="AK10" s="45" t="s">
         <v>90</v>
       </c>
-      <c r="AM10" s="48"/>
-      <c r="AN10" s="47"/>
-      <c r="AO10" s="47"/>
-      <c r="AP10" s="47"/>
-      <c r="AQ10" s="47"/>
-      <c r="AR10" s="47"/>
-      <c r="AS10" s="47"/>
-      <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
-      <c r="AW10" s="46"/>
+      <c r="AM10" s="100"/>
+      <c r="AN10" s="101"/>
+      <c r="AO10" s="101"/>
+      <c r="AP10" s="101"/>
+      <c r="AQ10" s="101"/>
+      <c r="AR10" s="101"/>
+      <c r="AS10" s="101"/>
+      <c r="AT10" s="101"/>
+      <c r="AU10" s="101"/>
+      <c r="AV10" s="101"/>
+      <c r="AW10" s="102"/>
       <c r="AZ10" s="13"/>
       <c r="BA10" s="13"/>
       <c r="BB10" s="13"/>
       <c r="BC10" s="13"/>
       <c r="BD10" s="13"/>
       <c r="BE10" s="13"/>
-      <c r="BF10" s="45">
+      <c r="BF10" s="44">
         <f>SUM(BF5:BF7)*BI5</f>
         <v>13676.25</v>
       </c>
       <c r="BG10" s="13"/>
-      <c r="BH10" s="44">
+      <c r="BH10" s="43">
         <v>170647.75</v>
       </c>
       <c r="BI10" s="13"/>
-      <c r="BJ10" s="43">
+      <c r="BJ10" s="42">
         <f>SUM(BJ5:BJ8)</f>
         <v>140269.5</v>
       </c>
@@ -2860,7 +2920,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="2:88" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:88" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>88</v>
       </c>
@@ -2875,7 +2935,7 @@
       <c r="I11" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="J11" s="42">
+      <c r="J11" s="41">
         <v>46113</v>
       </c>
       <c r="K11" s="1"/>
@@ -2898,7 +2958,7 @@
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
       <c r="X11" s="1"/>
-      <c r="AG11" s="41"/>
+      <c r="AG11" s="111"/>
       <c r="AH11" s="40"/>
       <c r="AI11" s="40"/>
       <c r="AJ11" s="40"/>
@@ -2961,7 +3021,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="2:88" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>80</v>
       </c>
@@ -3057,7 +3117,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="2:88" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>71</v>
       </c>
@@ -3162,7 +3222,7 @@
         <v>1800</v>
       </c>
     </row>
-    <row r="14" spans="2:88" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>59</v>
       </c>
@@ -3253,7 +3313,7 @@
       </c>
       <c r="CF14" s="27"/>
     </row>
-    <row r="15" spans="2:88" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>50</v>
       </c>
@@ -3332,7 +3392,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="2:88" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:88" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>43</v>
       </c>
@@ -3391,7 +3451,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:74" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>40</v>
       </c>
@@ -3448,7 +3508,7 @@
       </c>
       <c r="BV17" s="1"/>
     </row>
-    <row r="18" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:74" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>37</v>
       </c>
@@ -3493,7 +3553,7 @@
       <c r="BU18" s="1"/>
       <c r="BV18" s="1"/>
     </row>
-    <row r="19" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:74" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>36</v>
       </c>
@@ -3546,7 +3606,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:74" x14ac:dyDescent="0.3">
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -3578,7 +3638,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:74" x14ac:dyDescent="0.3">
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -3610,7 +3670,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:74" x14ac:dyDescent="0.3">
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -3642,7 +3702,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="2:74" ht="19" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:74" ht="18" x14ac:dyDescent="0.35">
+      <c r="O23" s="118" t="s">
+        <v>207</v>
+      </c>
+      <c r="P23" s="118"/>
+      <c r="Q23" s="118"/>
+      <c r="R23" s="118"/>
       <c r="S23" s="12"/>
       <c r="U23" s="10" t="s">
         <v>28</v>
@@ -3664,7 +3730,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:74" ht="19" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:74" ht="19.05" customHeight="1" x14ac:dyDescent="0.5">
       <c r="E24" s="9">
         <f>SUM(E6:E19)</f>
         <v>58960</v>
@@ -3699,7 +3765,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:74" x14ac:dyDescent="0.3">
       <c r="BT25" s="1" t="s">
         <v>23</v>
       </c>
@@ -3710,7 +3776,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="2:74" ht="26" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:74" ht="25.8" x14ac:dyDescent="0.5">
       <c r="U26" s="7">
         <f>U24-W24</f>
         <v>157133.96</v>
@@ -3730,7 +3796,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:74" x14ac:dyDescent="0.3">
       <c r="BT27" s="1"/>
       <c r="BU27" s="2">
         <f>SUM(BU19:BU26)</f>
@@ -3738,13 +3804,13 @@
       </c>
       <c r="BV27" s="1"/>
     </row>
-    <row r="28" spans="2:74" ht="26" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:74" ht="25.8" x14ac:dyDescent="0.5">
       <c r="X28" s="6"/>
       <c r="BT28" s="1"/>
       <c r="BU28" s="1"/>
       <c r="BV28" s="1"/>
     </row>
-    <row r="29" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:74" x14ac:dyDescent="0.3">
       <c r="BT29" s="1" t="s">
         <v>21</v>
       </c>
@@ -3755,7 +3821,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:74" x14ac:dyDescent="0.3">
       <c r="W30" t="s">
         <v>20</v>
       </c>
@@ -3772,7 +3838,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:74" x14ac:dyDescent="0.3">
       <c r="W31" t="s">
         <v>18</v>
       </c>
@@ -3786,7 +3852,7 @@
       </c>
       <c r="BV31" s="1"/>
     </row>
-    <row r="32" spans="2:74" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:74" x14ac:dyDescent="0.3">
       <c r="W32" t="s">
         <v>17</v>
       </c>
@@ -3797,7 +3863,7 @@
       <c r="BU32" s="1"/>
       <c r="BV32" s="1"/>
     </row>
-    <row r="33" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="33" spans="23:74" x14ac:dyDescent="0.3">
       <c r="W33" t="s">
         <v>16</v>
       </c>
@@ -3810,7 +3876,7 @@
       <c r="BU33" s="1"/>
       <c r="BV33" s="1"/>
     </row>
-    <row r="34" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="34" spans="23:74" x14ac:dyDescent="0.3">
       <c r="W34" t="s">
         <v>14</v>
       </c>
@@ -3827,7 +3893,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="35" spans="23:74" x14ac:dyDescent="0.3">
       <c r="W35" t="s">
         <v>12</v>
       </c>
@@ -3844,7 +3910,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="36" spans="23:74" x14ac:dyDescent="0.3">
       <c r="W36" t="s">
         <v>10</v>
       </c>
@@ -3861,7 +3927,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="37" spans="23:74" x14ac:dyDescent="0.3">
       <c r="BT37" s="1"/>
       <c r="BU37" s="2">
         <f>SUM(BU34:BU36)</f>
@@ -3869,7 +3935,7 @@
       </c>
       <c r="BV37" s="1"/>
     </row>
-    <row r="38" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="38" spans="23:74" x14ac:dyDescent="0.3">
       <c r="X38" s="5">
         <f>SUM(X30:X37)</f>
         <v>7710</v>
@@ -3878,7 +3944,7 @@
       <c r="BU38" s="1"/>
       <c r="BV38" s="1"/>
     </row>
-    <row r="39" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="39" spans="23:74" x14ac:dyDescent="0.3">
       <c r="X39" s="3">
         <f>X24-70000</f>
         <v>16781.75</v>
@@ -3893,7 +3959,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="40" spans="23:74" x14ac:dyDescent="0.3">
       <c r="X40" s="4">
         <f>X39-X38</f>
         <v>9071.75</v>
@@ -3908,7 +3974,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="41" spans="23:74" x14ac:dyDescent="0.3">
       <c r="X41" s="3">
         <f>X40-3000</f>
         <v>6071.75</v>
@@ -3923,7 +3989,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="42" spans="23:74" x14ac:dyDescent="0.3">
       <c r="BT42" s="1" t="s">
         <v>4</v>
       </c>
@@ -3934,7 +4000,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="43" spans="23:74" x14ac:dyDescent="0.3">
       <c r="BT43" s="1" t="s">
         <v>3</v>
       </c>
@@ -3945,7 +4011,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="44" spans="23:74" x14ac:dyDescent="0.3">
       <c r="BT44" s="1"/>
       <c r="BU44" s="2">
         <f>SUM(BU39:BU43)</f>
@@ -3953,12 +4019,12 @@
       </c>
       <c r="BV44" s="1"/>
     </row>
-    <row r="45" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="45" spans="23:74" x14ac:dyDescent="0.3">
       <c r="BT45" s="1"/>
       <c r="BU45" s="2"/>
       <c r="BV45" s="1"/>
     </row>
-    <row r="46" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="46" spans="23:74" x14ac:dyDescent="0.3">
       <c r="BT46" s="1" t="s">
         <v>1</v>
       </c>
@@ -3967,12 +4033,12 @@
       </c>
       <c r="BV46" s="1"/>
     </row>
-    <row r="47" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="47" spans="23:74" x14ac:dyDescent="0.3">
       <c r="BT47" s="1"/>
       <c r="BU47" s="1"/>
       <c r="BV47" s="1"/>
     </row>
-    <row r="48" spans="23:74" x14ac:dyDescent="0.2">
+    <row r="48" spans="23:74" x14ac:dyDescent="0.3">
       <c r="BT48" s="2" t="s">
         <v>0</v>
       </c>
@@ -3983,7 +4049,10 @@
       <c r="BV48" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="10">
+    <mergeCell ref="AN3:AV3"/>
+    <mergeCell ref="N1:O3"/>
+    <mergeCell ref="O23:R23"/>
     <mergeCell ref="AM10:AW10"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="I4:M4"/>

</xml_diff>